<commit_message>
feat: add leaderboard screen and stabilize bgm flow
</commit_message>
<xml_diff>
--- a/docs/audio_catalog.xlsx
+++ b/docs/audio_catalog.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -521,7 +521,11 @@
           <t>主選單背景音樂</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>music_mainMenu.m4a</t>
+        </is>
+      </c>
       <c r="E2" t="inlineStr">
         <is>
           <t>home</t>
@@ -533,8 +537,6 @@
       <c r="G2" t="b">
         <v>1</v>
       </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
           <t>all</t>
@@ -545,7 +547,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>對應主畫面</t>
+          <t>主選單實際音檔（wav -&gt; m4a 已轉檔接入）</t>
         </is>
       </c>
     </row>
@@ -565,7 +567,6 @@
           <t>關卡選擇背景音樂</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>stageSelect</t>
@@ -577,8 +578,6 @@
       <c r="G3" t="b">
         <v>1</v>
       </c>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
           <t>all</t>
@@ -606,10 +605,14 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>戰鬥背景音樂</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
+          <t>一般關卡背景音樂</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>music_battle.m4a</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr">
         <is>
           <t>battle</t>
@@ -621,8 +624,6 @@
       <c r="G4" t="b">
         <v>1</v>
       </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
           <t>all</t>
@@ -633,7 +634,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>對應戰鬥</t>
+          <t>一般戰鬥音樂（已接入）</t>
         </is>
       </c>
     </row>
@@ -653,7 +654,11 @@
           <t>讀書強化背景音樂</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>music_researchPage.m4a</t>
+        </is>
+      </c>
       <c r="E5" t="inlineStr">
         <is>
           <t>study</t>
@@ -677,7 +682,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>對應讀書強化</t>
+          <t>讀書強化音樂（已接入）</t>
         </is>
       </c>
     </row>
@@ -697,7 +702,6 @@
           <t>設定背景音樂</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
           <t>settings</t>
@@ -709,8 +713,6 @@
       <c r="G6" t="b">
         <v>1</v>
       </c>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
           <t>all</t>
@@ -741,7 +743,6 @@
           <t>角色選擇背景音樂</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
           <t>characterSelect</t>
@@ -753,8 +754,6 @@
       <c r="G7" t="b">
         <v>1</v>
       </c>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr">
         <is>
           <t>all</t>
@@ -785,7 +784,6 @@
           <t>技能配置背景音樂</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
           <t>skillLoadout</t>
@@ -797,8 +795,6 @@
       <c r="G8" t="b">
         <v>1</v>
       </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
           <t>all</t>
@@ -845,8 +841,6 @@
       <c r="G9" t="b">
         <v>0</v>
       </c>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr">
         <is>
           <t>all</t>
@@ -877,7 +871,6 @@
           <t>散光斬施放音效</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
           <t>skill:astig</t>
@@ -889,8 +882,6 @@
       <c r="G10" t="b">
         <v>0</v>
       </c>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr">
         <is>
           <t>all</t>
@@ -921,7 +912,6 @@
           <t>黃斑殺施放音效</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
           <t>skill:macular</t>
@@ -933,8 +923,6 @@
       <c r="G11" t="b">
         <v>0</v>
       </c>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
           <t>all</t>
@@ -965,7 +953,6 @@
           <t>稜鏡破施放音效</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
           <t>skill:prism-break</t>
@@ -977,8 +964,6 @@
       <c r="G12" t="b">
         <v>0</v>
       </c>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr">
         <is>
           <t>all</t>
@@ -1009,7 +994,6 @@
           <t>閃光眼施放音效</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
           <t>skill:flash-glare</t>
@@ -1021,8 +1005,6 @@
       <c r="G13" t="b">
         <v>0</v>
       </c>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr">
         <is>
           <t>all</t>
@@ -1053,7 +1035,6 @@
           <t>全視野掃描施放音效</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
           <t>skill:full-field-scan</t>
@@ -1065,8 +1046,6 @@
       <c r="G14" t="b">
         <v>0</v>
       </c>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr">
         <is>
           <t>all</t>
@@ -1078,6 +1057,52 @@
       <c r="L14" t="inlineStr">
         <is>
           <t>待提供音檔</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>bgm_battle_boss</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>bgm</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Boss 關卡背景音樂</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>music_battleWithBoss.m4a</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>battleBoss</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G15" t="b">
+        <v>1</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="K15" t="b">
+        <v>1</v>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Boss 戰鬥音樂（已接入）</t>
         </is>
       </c>
     </row>

</xml_diff>